<commit_message>
Fixed formatting errors in cycle document.
</commit_message>
<xml_diff>
--- a/Research/Instructions/Ricoh 5A22 Instructions Emulation SNES.xlsx
+++ b/Research/Instructions/Ricoh 5A22 Instructions Emulation SNES.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\My Projects\BirdSNES\Research\Instructions\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4FEE5B5-15AA-40C4-BE9A-9C7689BF4152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B99E027D-5A34-4539-A70D-49A0071B6761}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{7ED93F2B-FF78-48E4-8428-9E2E36877943}"/>
   </bookViews>
@@ -14268,17 +14268,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -14884,10 +14884,10 @@
     </row>
     <row r="61" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>
-      <c r="B61" s="36" t="s">
+      <c r="B61" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C61" s="37"/>
+      <c r="C61" s="39"/>
     </row>
     <row r="62" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="12" t="s">
@@ -15008,7 +15008,7 @@
       <c r="A75" s="8">
         <v>5.2</v>
       </c>
-      <c r="B75" s="38" t="s">
+      <c r="B75" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C75" s="14" t="s">
@@ -15017,12 +15017,12 @@
     </row>
     <row r="76" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="8"/>
-      <c r="B76" s="38"/>
+      <c r="B76" s="37"/>
       <c r="C76" s="14"/>
     </row>
     <row r="77" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="8"/>
-      <c r="B77" s="38"/>
+      <c r="B77" s="37"/>
       <c r="C77" s="14"/>
     </row>
     <row r="78" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -15308,10 +15308,10 @@
     </row>
     <row r="179" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A179" s="4"/>
-      <c r="B179" s="36" t="s">
+      <c r="B179" s="38" t="s">
         <v>55</v>
       </c>
-      <c r="C179" s="37"/>
+      <c r="C179" s="39"/>
     </row>
     <row r="180" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A180" s="12" t="s">
@@ -15817,14 +15817,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B367" s="9"/>
-      <c r="C367" s="39" t="s">
+      <c r="C367" s="36" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="368" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A368" s="8"/>
       <c r="B368" s="9"/>
-      <c r="C368" s="39"/>
+      <c r="C368" s="36"/>
     </row>
     <row r="369" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A369" s="18">
@@ -15875,10 +15875,10 @@
     </row>
     <row r="415" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A415" s="4"/>
-      <c r="B415" s="36" t="s">
+      <c r="B415" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="C415" s="37"/>
+      <c r="C415" s="39"/>
     </row>
     <row r="416" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A416" s="12" t="s">
@@ -16446,10 +16446,10 @@
     </row>
     <row r="710" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A710" s="4"/>
-      <c r="B710" s="36" t="s">
+      <c r="B710" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C710" s="37"/>
+      <c r="C710" s="39"/>
     </row>
     <row r="711" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A711" s="12" t="s">
@@ -16736,10 +16736,10 @@
     </row>
     <row r="828" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A828" s="4"/>
-      <c r="B828" s="36" t="s">
+      <c r="B828" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C828" s="37"/>
+      <c r="C828" s="39"/>
     </row>
     <row r="829" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A829" s="12" t="s">
@@ -16846,14 +16846,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B839" s="9"/>
-      <c r="C839" s="39" t="s">
+      <c r="C839" s="36" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A840" s="8"/>
       <c r="B840" s="9"/>
-      <c r="C840" s="39"/>
+      <c r="C840" s="36"/>
     </row>
     <row r="841" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A841" s="18">
@@ -16904,10 +16904,10 @@
     </row>
     <row r="887" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A887" s="4"/>
-      <c r="B887" s="36" t="s">
+      <c r="B887" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="C887" s="37"/>
+      <c r="C887" s="39"/>
     </row>
     <row r="888" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A888" s="12" t="s">
@@ -17094,14 +17094,14 @@
       <c r="B950" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C950" s="39" t="s">
+      <c r="C950" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="951" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A951" s="8"/>
       <c r="B951" s="9"/>
-      <c r="C951" s="39"/>
+      <c r="C951" s="36"/>
     </row>
     <row r="952" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A952" s="8">
@@ -17177,10 +17177,10 @@
     </row>
     <row r="1005" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1005" s="4"/>
-      <c r="B1005" s="36" t="s">
+      <c r="B1005" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C1005" s="37"/>
+      <c r="C1005" s="39"/>
     </row>
     <row r="1006" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1006" s="12" t="s">
@@ -17380,10 +17380,10 @@
     </row>
     <row r="1064" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1064" s="4"/>
-      <c r="B1064" s="36" t="s">
+      <c r="B1064" s="38" t="s">
         <v>96</v>
       </c>
-      <c r="C1064" s="37"/>
+      <c r="C1064" s="39"/>
     </row>
     <row r="1065" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1065" s="12" t="s">
@@ -17539,10 +17539,10 @@
     </row>
     <row r="1123" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1123" s="4"/>
-      <c r="B1123" s="36" t="s">
+      <c r="B1123" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="C1123" s="37"/>
+      <c r="C1123" s="39"/>
     </row>
     <row r="1124" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1124" s="12" t="s">
@@ -17726,10 +17726,10 @@
     </row>
     <row r="1182" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1182" s="4"/>
-      <c r="B1182" s="36" t="s">
+      <c r="B1182" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="C1182" s="37"/>
+      <c r="C1182" s="39"/>
     </row>
     <row r="1183" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1183" s="12" t="s">
@@ -17953,14 +17953,14 @@
         <v>3.1</v>
       </c>
       <c r="B1248" s="9"/>
-      <c r="C1248" s="39" t="s">
+      <c r="C1248" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="1249" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1249" s="8"/>
       <c r="B1249" s="9"/>
-      <c r="C1249" s="39"/>
+      <c r="C1249" s="36"/>
     </row>
     <row r="1250" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1250" s="15">
@@ -18027,10 +18027,10 @@
     </row>
     <row r="1300" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1300" s="4"/>
-      <c r="B1300" s="36" t="s">
+      <c r="B1300" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="C1300" s="37"/>
+      <c r="C1300" s="39"/>
     </row>
     <row r="1301" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1301" s="12" t="s">
@@ -18095,14 +18095,14 @@
         <v>3.1</v>
       </c>
       <c r="B1307" s="9"/>
-      <c r="C1307" s="39" t="s">
+      <c r="C1307" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="1308" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1308" s="8"/>
       <c r="B1308" s="9"/>
-      <c r="C1308" s="39"/>
+      <c r="C1308" s="36"/>
     </row>
     <row r="1309" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1309" s="15">
@@ -18152,14 +18152,14 @@
         <v>6.1</v>
       </c>
       <c r="B1314" s="9"/>
-      <c r="C1314" s="39" t="s">
+      <c r="C1314" s="36" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="1315" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1315" s="8"/>
       <c r="B1315" s="9"/>
-      <c r="C1315" s="39"/>
+      <c r="C1315" s="36"/>
     </row>
     <row r="1316" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1316" s="18">
@@ -18210,10 +18210,10 @@
     </row>
     <row r="1359" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1359" s="4"/>
-      <c r="B1359" s="36" t="s">
+      <c r="B1359" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C1359" s="37"/>
+      <c r="C1359" s="39"/>
     </row>
     <row r="1360" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1360" s="12" t="s">
@@ -18304,7 +18304,7 @@
       <c r="A1369" s="8">
         <v>4.2</v>
       </c>
-      <c r="B1369" s="38" t="s">
+      <c r="B1369" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C1369" s="14" t="s">
@@ -18313,12 +18313,12 @@
     </row>
     <row r="1370" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1370" s="8"/>
-      <c r="B1370" s="38"/>
+      <c r="B1370" s="37"/>
       <c r="C1370" s="14"/>
     </row>
     <row r="1371" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1371" s="8"/>
-      <c r="B1371" s="38"/>
+      <c r="B1371" s="37"/>
       <c r="C1371" s="14"/>
     </row>
     <row r="1372" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18332,7 +18332,7 @@
       <c r="A1373" s="8">
         <v>5.2</v>
       </c>
-      <c r="B1373" s="38" t="s">
+      <c r="B1373" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C1373" s="10" t="s">
@@ -18341,12 +18341,12 @@
     </row>
     <row r="1374" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1374" s="8"/>
-      <c r="B1374" s="38"/>
+      <c r="B1374" s="37"/>
       <c r="C1374" s="10"/>
     </row>
     <row r="1375" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1375" s="8"/>
-      <c r="B1375" s="38"/>
+      <c r="B1375" s="37"/>
       <c r="C1375" s="10"/>
     </row>
     <row r="1376" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -18510,10 +18510,10 @@
     </row>
     <row r="1477" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1477" s="4"/>
-      <c r="B1477" s="36" t="s">
+      <c r="B1477" s="38" t="s">
         <v>114</v>
       </c>
-      <c r="C1477" s="37"/>
+      <c r="C1477" s="39"/>
     </row>
     <row r="1478" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1478" s="12" t="s">
@@ -18853,10 +18853,10 @@
     </row>
     <row r="1654" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1654" s="4"/>
-      <c r="B1654" s="36" t="s">
+      <c r="B1654" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C1654" s="37"/>
+      <c r="C1654" s="39"/>
     </row>
     <row r="1655" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1655" s="12" t="s">
@@ -19016,10 +19016,10 @@
     </row>
     <row r="1713" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1713" s="4"/>
-      <c r="B1713" s="36" t="s">
+      <c r="B1713" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="C1713" s="37"/>
+      <c r="C1713" s="39"/>
     </row>
     <row r="1714" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1714" s="12" t="s">
@@ -19185,10 +19185,10 @@
     </row>
     <row r="1772" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1772" s="4"/>
-      <c r="B1772" s="36" t="s">
+      <c r="B1772" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="C1772" s="37"/>
+      <c r="C1772" s="39"/>
     </row>
     <row r="1773" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1773" s="12" t="s">
@@ -19323,14 +19323,14 @@
         <v>6.1</v>
       </c>
       <c r="B1787" s="9"/>
-      <c r="C1787" s="39" t="s">
+      <c r="C1787" s="36" t="s">
         <v>146</v>
       </c>
     </row>
     <row r="1788" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1788" s="8"/>
       <c r="B1788" s="9"/>
-      <c r="C1788" s="39"/>
+      <c r="C1788" s="36"/>
     </row>
     <row r="1789" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1789" s="18">
@@ -19381,10 +19381,10 @@
     </row>
     <row r="1831" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1831" s="4"/>
-      <c r="B1831" s="36" t="s">
+      <c r="B1831" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="C1831" s="37"/>
+      <c r="C1831" s="39"/>
     </row>
     <row r="1832" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1832" s="12" t="s">
@@ -19542,10 +19542,10 @@
     </row>
     <row r="1890" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1890" s="4"/>
-      <c r="B1890" s="36" t="s">
+      <c r="B1890" s="38" t="s">
         <v>130</v>
       </c>
-      <c r="C1890" s="37"/>
+      <c r="C1890" s="39"/>
     </row>
     <row r="1891" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1891" s="12" t="s">
@@ -19707,10 +19707,10 @@
     </row>
     <row r="1949" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1949" s="4"/>
-      <c r="B1949" s="36" t="s">
+      <c r="B1949" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C1949" s="37"/>
+      <c r="C1949" s="39"/>
     </row>
     <row r="1950" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1950" s="12" t="s">
@@ -19831,7 +19831,7 @@
       <c r="A1963" s="8">
         <v>5.2</v>
       </c>
-      <c r="B1963" s="38" t="s">
+      <c r="B1963" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C1963" s="14" t="s">
@@ -19840,12 +19840,12 @@
     </row>
     <row r="1964" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1964" s="8"/>
-      <c r="B1964" s="38"/>
+      <c r="B1964" s="37"/>
       <c r="C1964" s="14"/>
     </row>
     <row r="1965" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1965" s="8"/>
-      <c r="B1965" s="38"/>
+      <c r="B1965" s="37"/>
       <c r="C1965" s="14"/>
     </row>
     <row r="1966" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -20477,10 +20477,10 @@
     </row>
     <row r="2244" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2244" s="4"/>
-      <c r="B2244" s="36" t="s">
+      <c r="B2244" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="C2244" s="37"/>
+      <c r="C2244" s="39"/>
     </row>
     <row r="2245" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2245" s="12" t="s">
@@ -20583,14 +20583,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B2255" s="9"/>
-      <c r="C2255" s="39" t="s">
+      <c r="C2255" s="36" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="2256" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2256" s="8"/>
       <c r="B2256" s="9"/>
-      <c r="C2256" s="39"/>
+      <c r="C2256" s="36"/>
     </row>
     <row r="2257" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2257" s="18">
@@ -21369,10 +21369,10 @@
     </row>
     <row r="2657" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2657" s="4"/>
-      <c r="B2657" s="36" t="s">
+      <c r="B2657" s="38" t="s">
         <v>29</v>
       </c>
-      <c r="C2657" s="37"/>
+      <c r="C2657" s="39"/>
     </row>
     <row r="2658" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2658" s="12" t="s">
@@ -21496,10 +21496,10 @@
     </row>
     <row r="2716" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2716" s="4"/>
-      <c r="B2716" s="36" t="s">
+      <c r="B2716" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C2716" s="37"/>
+      <c r="C2716" s="39"/>
     </row>
     <row r="2717" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2717" s="12" t="s">
@@ -21606,14 +21606,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B2727" s="9"/>
-      <c r="C2727" s="39" t="s">
+      <c r="C2727" s="36" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="2728" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2728" s="8"/>
       <c r="B2728" s="9"/>
-      <c r="C2728" s="39"/>
+      <c r="C2728" s="36"/>
     </row>
     <row r="2729" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2729" s="18">
@@ -21664,10 +21664,10 @@
     </row>
     <row r="2775" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2775" s="4"/>
-      <c r="B2775" s="36" t="s">
+      <c r="B2775" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="C2775" s="37"/>
+      <c r="C2775" s="39"/>
     </row>
     <row r="2776" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2776" s="12" t="s">
@@ -21854,14 +21854,14 @@
       <c r="B2838" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C2838" s="39" t="s">
+      <c r="C2838" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="2839" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2839" s="8"/>
       <c r="B2839" s="9"/>
-      <c r="C2839" s="39"/>
+      <c r="C2839" s="36"/>
     </row>
     <row r="2840" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2840" s="8">
@@ -21937,10 +21937,10 @@
     </row>
     <row r="2893" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2893" s="4"/>
-      <c r="B2893" s="36" t="s">
+      <c r="B2893" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C2893" s="37"/>
+      <c r="C2893" s="39"/>
     </row>
     <row r="2894" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2894" s="12" t="s">
@@ -22299,10 +22299,10 @@
     </row>
     <row r="3011" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3011" s="4"/>
-      <c r="B3011" s="36" t="s">
+      <c r="B3011" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="C3011" s="37"/>
+      <c r="C3011" s="39"/>
     </row>
     <row r="3012" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3012" s="12" t="s">
@@ -22554,14 +22554,14 @@
         <v>3.1</v>
       </c>
       <c r="B3077" s="9"/>
-      <c r="C3077" s="39" t="s">
+      <c r="C3077" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="3078" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3078" s="8"/>
       <c r="B3078" s="9"/>
-      <c r="C3078" s="39"/>
+      <c r="C3078" s="36"/>
     </row>
     <row r="3079" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3079" s="15">
@@ -22706,14 +22706,14 @@
         <v>3.1</v>
       </c>
       <c r="B3136" s="9"/>
-      <c r="C3136" s="39" t="s">
+      <c r="C3136" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="3137" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3137" s="8"/>
       <c r="B3137" s="9"/>
-      <c r="C3137" s="39"/>
+      <c r="C3137" s="36"/>
     </row>
     <row r="3138" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3138" s="15">
@@ -22780,10 +22780,10 @@
     </row>
     <row r="3188" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3188" s="4"/>
-      <c r="B3188" s="36" t="s">
+      <c r="B3188" s="38" t="s">
         <v>107</v>
       </c>
-      <c r="C3188" s="37"/>
+      <c r="C3188" s="39"/>
     </row>
     <row r="3189" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3189" s="12" t="s">
@@ -22848,14 +22848,14 @@
         <v>3.1</v>
       </c>
       <c r="B3195" s="9"/>
-      <c r="C3195" s="39" t="s">
+      <c r="C3195" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="3196" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3196" s="8"/>
       <c r="B3196" s="9"/>
-      <c r="C3196" s="39"/>
+      <c r="C3196" s="36"/>
     </row>
     <row r="3197" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3197" s="15">
@@ -22905,14 +22905,14 @@
         <v>6.1</v>
       </c>
       <c r="B3202" s="9"/>
-      <c r="C3202" s="39" t="s">
+      <c r="C3202" s="36" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="3203" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3203" s="8"/>
       <c r="B3203" s="9"/>
-      <c r="C3203" s="39"/>
+      <c r="C3203" s="36"/>
     </row>
     <row r="3204" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3204" s="18">
@@ -22973,10 +22973,10 @@
     </row>
     <row r="3247" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3247" s="4"/>
-      <c r="B3247" s="36" t="s">
+      <c r="B3247" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C3247" s="37"/>
+      <c r="C3247" s="39"/>
     </row>
     <row r="3248" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3248" s="12" t="s">
@@ -23067,7 +23067,7 @@
       <c r="A3257" s="8">
         <v>4.2</v>
       </c>
-      <c r="B3257" s="38" t="s">
+      <c r="B3257" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C3257" s="10" t="s">
@@ -23076,12 +23076,12 @@
     </row>
     <row r="3258" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3258" s="8"/>
-      <c r="B3258" s="38"/>
+      <c r="B3258" s="37"/>
       <c r="C3258" s="10"/>
     </row>
     <row r="3259" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3259" s="8"/>
-      <c r="B3259" s="38"/>
+      <c r="B3259" s="37"/>
       <c r="C3259" s="10"/>
     </row>
     <row r="3260" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -23095,7 +23095,7 @@
       <c r="A3261" s="8">
         <v>5.2</v>
       </c>
-      <c r="B3261" s="38" t="s">
+      <c r="B3261" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C3261" s="10" t="s">
@@ -23104,12 +23104,12 @@
     </row>
     <row r="3262" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3262" s="8"/>
-      <c r="B3262" s="38"/>
+      <c r="B3262" s="37"/>
       <c r="C3262" s="10"/>
     </row>
     <row r="3263" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3263" s="8"/>
-      <c r="B3263" s="38"/>
+      <c r="B3263" s="37"/>
       <c r="C3263" s="10"/>
     </row>
     <row r="3264" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -23273,10 +23273,10 @@
     </row>
     <row r="3365" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3365" s="4"/>
-      <c r="B3365" s="36" t="s">
+      <c r="B3365" s="38" t="s">
         <v>114</v>
       </c>
-      <c r="C3365" s="37"/>
+      <c r="C3365" s="39"/>
     </row>
     <row r="3366" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3366" s="12" t="s">
@@ -23954,10 +23954,10 @@
     </row>
     <row r="3660" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3660" s="4"/>
-      <c r="B3660" s="36" t="s">
+      <c r="B3660" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="C3660" s="37"/>
+      <c r="C3660" s="39"/>
     </row>
     <row r="3661" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3661" s="12" t="s">
@@ -24092,14 +24092,14 @@
         <v>6.1</v>
       </c>
       <c r="B3675" s="9"/>
-      <c r="C3675" s="39" t="s">
+      <c r="C3675" s="36" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="3676" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3676" s="8"/>
       <c r="B3676" s="9"/>
-      <c r="C3676" s="39"/>
+      <c r="C3676" s="36"/>
     </row>
     <row r="3677" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3677" s="18">
@@ -24466,10 +24466,10 @@
     </row>
     <row r="3837" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3837" s="4"/>
-      <c r="B3837" s="36" t="s">
+      <c r="B3837" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C3837" s="37"/>
+      <c r="C3837" s="39"/>
     </row>
     <row r="3838" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3838" s="12" t="s">
@@ -24590,7 +24590,7 @@
       <c r="A3851" s="8">
         <v>5.2</v>
       </c>
-      <c r="B3851" s="38" t="s">
+      <c r="B3851" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C3851" s="14" t="s">
@@ -24599,12 +24599,12 @@
     </row>
     <row r="3852" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3852" s="8"/>
-      <c r="B3852" s="38"/>
+      <c r="B3852" s="37"/>
       <c r="C3852" s="14"/>
     </row>
     <row r="3853" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3853" s="8"/>
-      <c r="B3853" s="38"/>
+      <c r="B3853" s="37"/>
       <c r="C3853" s="14"/>
     </row>
     <row r="3854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -24670,10 +24670,10 @@
     </row>
     <row r="3896" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3896" s="4"/>
-      <c r="B3896" s="36" t="s">
+      <c r="B3896" s="38" t="s">
         <v>34</v>
       </c>
-      <c r="C3896" s="37"/>
+      <c r="C3896" s="39"/>
     </row>
     <row r="3897" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3897" s="12" t="s">
@@ -24878,10 +24878,10 @@
     </row>
     <row r="4014" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4014" s="4"/>
-      <c r="B4014" s="36" t="s">
+      <c r="B4014" s="38" t="s">
         <v>242</v>
       </c>
-      <c r="C4014" s="37"/>
+      <c r="C4014" s="39"/>
     </row>
     <row r="4015" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4015" s="12" t="s">
@@ -24988,14 +24988,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B4025" s="9"/>
-      <c r="C4025" s="39" t="s">
+      <c r="C4025" s="36" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="4026" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4026" s="8"/>
       <c r="B4026" s="9"/>
-      <c r="C4026" s="39"/>
+      <c r="C4026" s="36"/>
     </row>
     <row r="4027" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4027" s="8">
@@ -25179,10 +25179,10 @@
     </row>
     <row r="4132" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4132" s="4"/>
-      <c r="B4132" s="36" t="s">
+      <c r="B4132" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="C4132" s="37"/>
+      <c r="C4132" s="39"/>
     </row>
     <row r="4133" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4133" s="12" t="s">
@@ -25285,14 +25285,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B4143" s="9"/>
-      <c r="C4143" s="39" t="s">
+      <c r="C4143" s="36" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="4144" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4144" s="8"/>
       <c r="B4144" s="9"/>
-      <c r="C4144" s="39"/>
+      <c r="C4144" s="36"/>
     </row>
     <row r="4145" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4145" s="18">
@@ -25343,10 +25343,10 @@
     </row>
     <row r="4191" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4191" s="4"/>
-      <c r="B4191" s="36" t="s">
+      <c r="B4191" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="C4191" s="37"/>
+      <c r="C4191" s="39"/>
     </row>
     <row r="4192" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4192" s="12" t="s">
@@ -26130,10 +26130,10 @@
     </row>
     <row r="4604" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4604" s="4"/>
-      <c r="B4604" s="36" t="s">
+      <c r="B4604" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C4604" s="37"/>
+      <c r="C4604" s="39"/>
     </row>
     <row r="4605" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4605" s="12" t="s">
@@ -26240,14 +26240,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B4615" s="9"/>
-      <c r="C4615" s="39" t="s">
+      <c r="C4615" s="36" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="4616" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4616" s="8"/>
       <c r="B4616" s="9"/>
-      <c r="C4616" s="39"/>
+      <c r="C4616" s="36"/>
     </row>
     <row r="4617" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4617" s="18">
@@ -26298,10 +26298,10 @@
     </row>
     <row r="4663" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4663" s="4"/>
-      <c r="B4663" s="36" t="s">
+      <c r="B4663" s="38" t="s">
         <v>83</v>
       </c>
-      <c r="C4663" s="37"/>
+      <c r="C4663" s="39"/>
     </row>
     <row r="4664" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4664" s="12" t="s">
@@ -26488,14 +26488,14 @@
       <c r="B4726" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C4726" s="39" t="s">
+      <c r="C4726" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="4727" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4727" s="8"/>
       <c r="B4727" s="9"/>
-      <c r="C4727" s="39"/>
+      <c r="C4727" s="36"/>
     </row>
     <row r="4728" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4728" s="8">
@@ -26571,10 +26571,10 @@
     </row>
     <row r="4781" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4781" s="4"/>
-      <c r="B4781" s="36" t="s">
+      <c r="B4781" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C4781" s="37"/>
+      <c r="C4781" s="39"/>
     </row>
     <row r="4782" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4782" s="12" t="s">
@@ -26926,10 +26926,10 @@
     </row>
     <row r="4899" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4899" s="4"/>
-      <c r="B4899" s="36" t="s">
+      <c r="B4899" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="C4899" s="37"/>
+      <c r="C4899" s="39"/>
     </row>
     <row r="4900" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4900" s="12" t="s">
@@ -27223,14 +27223,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B4969" s="9"/>
-      <c r="C4969" s="39" t="s">
+      <c r="C4969" s="36" t="s">
         <v>249</v>
       </c>
     </row>
     <row r="4970" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4970" s="8"/>
       <c r="B4970" s="9"/>
-      <c r="C4970" s="39"/>
+      <c r="C4970" s="36"/>
     </row>
     <row r="4971" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4971" s="8">
@@ -27359,14 +27359,14 @@
         <v>3.1</v>
       </c>
       <c r="B5024" s="9"/>
-      <c r="C5024" s="39" t="s">
+      <c r="C5024" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5025" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5025" s="8"/>
       <c r="B5025" s="9"/>
-      <c r="C5025" s="39"/>
+      <c r="C5025" s="36"/>
     </row>
     <row r="5026" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5026" s="15">
@@ -27433,10 +27433,10 @@
     </row>
     <row r="5076" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5076" s="4"/>
-      <c r="B5076" s="36" t="s">
+      <c r="B5076" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="C5076" s="37"/>
+      <c r="C5076" s="39"/>
     </row>
     <row r="5077" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5077" s="12" t="s">
@@ -27501,14 +27501,14 @@
         <v>3.1</v>
       </c>
       <c r="B5083" s="9"/>
-      <c r="C5083" s="39" t="s">
+      <c r="C5083" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="5084" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5084" s="8"/>
       <c r="B5084" s="9"/>
-      <c r="C5084" s="39"/>
+      <c r="C5084" s="36"/>
     </row>
     <row r="5085" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5085" s="15">
@@ -27558,14 +27558,14 @@
         <v>6.1</v>
       </c>
       <c r="B5090" s="9"/>
-      <c r="C5090" s="39" t="s">
+      <c r="C5090" s="36" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="5091" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5091" s="8"/>
       <c r="B5091" s="9"/>
-      <c r="C5091" s="39"/>
+      <c r="C5091" s="36"/>
     </row>
     <row r="5092" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5092" s="18">
@@ -27616,10 +27616,10 @@
     </row>
     <row r="5135" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5135" s="4"/>
-      <c r="B5135" s="36" t="s">
+      <c r="B5135" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C5135" s="37"/>
+      <c r="C5135" s="39"/>
     </row>
     <row r="5136" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5136" s="12" t="s">
@@ -27710,7 +27710,7 @@
       <c r="A5145" s="8">
         <v>4.2</v>
       </c>
-      <c r="B5145" s="38" t="s">
+      <c r="B5145" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C5145" s="10" t="s">
@@ -27719,12 +27719,12 @@
     </row>
     <row r="5146" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5146" s="8"/>
-      <c r="B5146" s="38"/>
+      <c r="B5146" s="37"/>
       <c r="C5146" s="10"/>
     </row>
     <row r="5147" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5147" s="8"/>
-      <c r="B5147" s="38"/>
+      <c r="B5147" s="37"/>
       <c r="C5147" s="10"/>
     </row>
     <row r="5148" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -27738,7 +27738,7 @@
       <c r="A5149" s="8">
         <v>5.2</v>
       </c>
-      <c r="B5149" s="38" t="s">
+      <c r="B5149" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C5149" s="10" t="s">
@@ -27747,12 +27747,12 @@
     </row>
     <row r="5150" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5150" s="8"/>
-      <c r="B5150" s="38"/>
+      <c r="B5150" s="37"/>
       <c r="C5150" s="10"/>
     </row>
     <row r="5151" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5151" s="8"/>
-      <c r="B5151" s="38"/>
+      <c r="B5151" s="37"/>
       <c r="C5151" s="10"/>
     </row>
     <row r="5152" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -28273,10 +28273,10 @@
     </row>
     <row r="5430" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5430" s="4"/>
-      <c r="B5430" s="36" t="s">
+      <c r="B5430" s="38" t="s">
         <v>134</v>
       </c>
-      <c r="C5430" s="37"/>
+      <c r="C5430" s="39"/>
     </row>
     <row r="5431" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5431" s="12" t="s">
@@ -28400,10 +28400,10 @@
     </row>
     <row r="5489" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5489" s="4"/>
-      <c r="B5489" s="36" t="s">
+      <c r="B5489" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="C5489" s="37"/>
+      <c r="C5489" s="39"/>
     </row>
     <row r="5490" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5490" s="12" t="s">
@@ -28562,10 +28562,10 @@
     </row>
     <row r="5548" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5548" s="4"/>
-      <c r="B5548" s="36" t="s">
+      <c r="B5548" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="C5548" s="37"/>
+      <c r="C5548" s="39"/>
     </row>
     <row r="5549" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5549" s="12" t="s">
@@ -28700,14 +28700,14 @@
         <v>6.1</v>
       </c>
       <c r="B5563" s="9"/>
-      <c r="C5563" s="39" t="s">
+      <c r="C5563" s="36" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="5564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5564" s="8"/>
       <c r="B5564" s="9"/>
-      <c r="C5564" s="39"/>
+      <c r="C5564" s="36"/>
     </row>
     <row r="5565" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5565" s="18">
@@ -28758,10 +28758,10 @@
     </row>
     <row r="5607" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5607" s="4"/>
-      <c r="B5607" s="36" t="s">
+      <c r="B5607" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="C5607" s="37"/>
+      <c r="C5607" s="39"/>
     </row>
     <row r="5608" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5608" s="12" t="s">
@@ -29068,10 +29068,10 @@
     </row>
     <row r="5725" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5725" s="4"/>
-      <c r="B5725" s="36" t="s">
+      <c r="B5725" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C5725" s="37"/>
+      <c r="C5725" s="39"/>
     </row>
     <row r="5726" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5726" s="12" t="s">
@@ -29192,7 +29192,7 @@
       <c r="A5739" s="8">
         <v>5.2</v>
       </c>
-      <c r="B5739" s="38" t="s">
+      <c r="B5739" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C5739" s="10" t="s">
@@ -29201,12 +29201,12 @@
     </row>
     <row r="5740" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5740" s="8"/>
-      <c r="B5740" s="38"/>
+      <c r="B5740" s="37"/>
       <c r="C5740" s="10"/>
     </row>
     <row r="5741" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5741" s="8"/>
-      <c r="B5741" s="38"/>
+      <c r="B5741" s="37"/>
       <c r="C5741" s="10"/>
     </row>
     <row r="5742" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -29370,10 +29370,10 @@
     </row>
     <row r="5784" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5784" s="4"/>
-      <c r="B5784" s="36" t="s">
+      <c r="B5784" s="38" t="s">
         <v>343</v>
       </c>
-      <c r="C5784" s="37"/>
+      <c r="C5784" s="39"/>
     </row>
     <row r="5785" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5785" s="12" t="s">
@@ -30090,10 +30090,10 @@
     </row>
     <row r="6020" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6020" s="4"/>
-      <c r="B6020" s="36" t="s">
+      <c r="B6020" s="38" t="s">
         <v>64</v>
       </c>
-      <c r="C6020" s="37"/>
+      <c r="C6020" s="39"/>
     </row>
     <row r="6021" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6021" s="12" t="s">
@@ -30196,14 +30196,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B6031" s="9"/>
-      <c r="C6031" s="39" t="s">
+      <c r="C6031" s="36" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="6032" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6032" s="8"/>
       <c r="B6032" s="9"/>
-      <c r="C6032" s="39"/>
+      <c r="C6032" s="36"/>
     </row>
     <row r="6033" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6033" s="18">
@@ -31439,10 +31439,10 @@
     </row>
     <row r="6492" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6492" s="4"/>
-      <c r="B6492" s="36" t="s">
+      <c r="B6492" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C6492" s="37"/>
+      <c r="C6492" s="39"/>
     </row>
     <row r="6493" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6493" s="12" t="s">
@@ -31549,14 +31549,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B6503" s="9"/>
-      <c r="C6503" s="39" t="s">
+      <c r="C6503" s="36" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="6504" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6504" s="8"/>
       <c r="B6504" s="9"/>
-      <c r="C6504" s="39"/>
+      <c r="C6504" s="36"/>
     </row>
     <row r="6505" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6505" s="18">
@@ -31895,14 +31895,14 @@
       <c r="B6614" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C6614" s="39" t="s">
+      <c r="C6614" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="6615" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6615" s="8"/>
       <c r="B6615" s="9"/>
-      <c r="C6615" s="39"/>
+      <c r="C6615" s="36"/>
     </row>
     <row r="6616" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6616" s="8">
@@ -31978,10 +31978,10 @@
     </row>
     <row r="6669" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6669" s="4"/>
-      <c r="B6669" s="36" t="s">
+      <c r="B6669" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C6669" s="37"/>
+      <c r="C6669" s="39"/>
     </row>
     <row r="6670" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6670" s="12" t="s">
@@ -32536,10 +32536,10 @@
     </row>
     <row r="6787" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6787" s="4"/>
-      <c r="B6787" s="36" t="s">
+      <c r="B6787" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="C6787" s="37"/>
+      <c r="C6787" s="39"/>
     </row>
     <row r="6788" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6788" s="12" t="s">
@@ -32889,14 +32889,14 @@
         <v>3.1</v>
       </c>
       <c r="B6853" s="9"/>
-      <c r="C6853" s="39" t="s">
+      <c r="C6853" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="6854" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6854" s="8"/>
       <c r="B6854" s="9"/>
-      <c r="C6854" s="39"/>
+      <c r="C6854" s="36"/>
     </row>
     <row r="6855" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6855" s="8">
@@ -33029,14 +33029,14 @@
         <v>3.1</v>
       </c>
       <c r="B6912" s="9"/>
-      <c r="C6912" s="39" t="s">
+      <c r="C6912" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="6913" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6913" s="8"/>
       <c r="B6913" s="9"/>
-      <c r="C6913" s="39"/>
+      <c r="C6913" s="36"/>
     </row>
     <row r="6914" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6914" s="8">
@@ -33201,10 +33201,10 @@
     </row>
     <row r="6964" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6964" s="4"/>
-      <c r="B6964" s="36" t="s">
+      <c r="B6964" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="C6964" s="37"/>
+      <c r="C6964" s="39"/>
     </row>
     <row r="6965" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6965" s="12" t="s">
@@ -33269,14 +33269,14 @@
         <v>3.1</v>
       </c>
       <c r="B6971" s="9"/>
-      <c r="C6971" s="39" t="s">
+      <c r="C6971" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="6972" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6972" s="8"/>
       <c r="B6972" s="9"/>
-      <c r="C6972" s="39"/>
+      <c r="C6972" s="36"/>
     </row>
     <row r="6973" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6973" s="8">
@@ -33326,14 +33326,14 @@
         <v>6.1</v>
       </c>
       <c r="B6978" s="9"/>
-      <c r="C6978" s="39" t="s">
+      <c r="C6978" s="36" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="6979" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6979" s="8"/>
       <c r="B6979" s="9"/>
-      <c r="C6979" s="39"/>
+      <c r="C6979" s="36"/>
     </row>
     <row r="6980" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6980" s="18">
@@ -33384,10 +33384,10 @@
     </row>
     <row r="7023" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7023" s="4"/>
-      <c r="B7023" s="36" t="s">
+      <c r="B7023" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C7023" s="37"/>
+      <c r="C7023" s="39"/>
     </row>
     <row r="7024" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7024" s="12" t="s">
@@ -33478,7 +33478,7 @@
       <c r="A7033" s="8">
         <v>4.2</v>
       </c>
-      <c r="B7033" s="38" t="s">
+      <c r="B7033" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C7033" s="10" t="s">
@@ -33487,12 +33487,12 @@
     </row>
     <row r="7034" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7034" s="8"/>
-      <c r="B7034" s="38"/>
+      <c r="B7034" s="37"/>
       <c r="C7034" s="10"/>
     </row>
     <row r="7035" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7035" s="8"/>
-      <c r="B7035" s="38"/>
+      <c r="B7035" s="37"/>
       <c r="C7035" s="10"/>
     </row>
     <row r="7036" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -33506,7 +33506,7 @@
       <c r="A7037" s="8">
         <v>5.2</v>
       </c>
-      <c r="B7037" s="38" t="s">
+      <c r="B7037" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C7037" s="10" t="s">
@@ -33515,12 +33515,12 @@
     </row>
     <row r="7038" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7038" s="8"/>
-      <c r="B7038" s="38"/>
+      <c r="B7038" s="37"/>
       <c r="C7038" s="10"/>
     </row>
     <row r="7039" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7039" s="8"/>
-      <c r="B7039" s="38"/>
+      <c r="B7039" s="37"/>
       <c r="C7039" s="10"/>
     </row>
     <row r="7040" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34130,19 +34130,19 @@
       <c r="A7209" s="8">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B7209" s="38" t="s">
+      <c r="B7209" s="37" t="s">
         <v>327</v>
       </c>
       <c r="C7209" s="10"/>
     </row>
     <row r="7210" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7210" s="8"/>
-      <c r="B7210" s="38"/>
+      <c r="B7210" s="37"/>
       <c r="C7210" s="10"/>
     </row>
     <row r="7211" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7211" s="8"/>
-      <c r="B7211" s="38"/>
+      <c r="B7211" s="37"/>
       <c r="C7211" s="10"/>
     </row>
     <row r="7212" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -34263,10 +34263,10 @@
     </row>
     <row r="7318" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7318" s="4"/>
-      <c r="B7318" s="36" t="s">
+      <c r="B7318" s="38" t="s">
         <v>498</v>
       </c>
-      <c r="C7318" s="37"/>
+      <c r="C7318" s="39"/>
     </row>
     <row r="7319" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7319" s="12" t="s">
@@ -34689,10 +34689,10 @@
     </row>
     <row r="7436" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7436" s="4"/>
-      <c r="B7436" s="36" t="s">
+      <c r="B7436" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="C7436" s="37"/>
+      <c r="C7436" s="39"/>
     </row>
     <row r="7437" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7437" s="12" t="s">
@@ -34827,14 +34827,14 @@
         <v>6.1</v>
       </c>
       <c r="B7451" s="27"/>
-      <c r="C7451" s="39" t="s">
+      <c r="C7451" s="36" t="s">
         <v>292</v>
       </c>
     </row>
     <row r="7452" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7452" s="8"/>
       <c r="B7452" s="27"/>
-      <c r="C7452" s="39"/>
+      <c r="C7452" s="36"/>
     </row>
     <row r="7453" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7453" s="18">
@@ -35187,14 +35187,14 @@
       <c r="B7558" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C7558" s="39" t="s">
+      <c r="C7558" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="7559" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7559" s="18"/>
       <c r="B7559" s="9"/>
-      <c r="C7559" s="39"/>
+      <c r="C7559" s="36"/>
     </row>
     <row r="7560" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7560" s="8">
@@ -35270,10 +35270,10 @@
     </row>
     <row r="7613" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7613" s="4"/>
-      <c r="B7613" s="36" t="s">
+      <c r="B7613" s="38" t="s">
         <v>339</v>
       </c>
-      <c r="C7613" s="37"/>
+      <c r="C7613" s="39"/>
     </row>
     <row r="7614" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7614" s="12" t="s">
@@ -35394,7 +35394,7 @@
       <c r="A7627" s="8">
         <v>5.2</v>
       </c>
-      <c r="B7627" s="38" t="s">
+      <c r="B7627" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C7627" s="10" t="s">
@@ -35403,12 +35403,12 @@
     </row>
     <row r="7628" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7628" s="8"/>
-      <c r="B7628" s="38"/>
+      <c r="B7628" s="37"/>
       <c r="C7628" s="10"/>
     </row>
     <row r="7629" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7629" s="8"/>
-      <c r="B7629" s="38"/>
+      <c r="B7629" s="37"/>
       <c r="C7629" s="10"/>
     </row>
     <row r="7630" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -35474,10 +35474,10 @@
     </row>
     <row r="7672" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7672" s="4"/>
-      <c r="B7672" s="36" t="s">
+      <c r="B7672" s="38" t="s">
         <v>343</v>
       </c>
-      <c r="C7672" s="37"/>
+      <c r="C7672" s="39"/>
     </row>
     <row r="7673" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7673" s="12" t="s">
@@ -37183,14 +37183,14 @@
       <c r="B8502" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C8502" s="39" t="s">
+      <c r="C8502" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="8503" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8503" s="8"/>
       <c r="B8503" s="9"/>
-      <c r="C8503" s="39"/>
+      <c r="C8503" s="36"/>
     </row>
     <row r="8504" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8504" s="8">
@@ -37266,10 +37266,10 @@
     </row>
     <row r="8557" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8557" s="4"/>
-      <c r="B8557" s="36" t="s">
+      <c r="B8557" s="38" t="s">
         <v>376</v>
       </c>
-      <c r="C8557" s="37"/>
+      <c r="C8557" s="39"/>
     </row>
     <row r="8558" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8558" s="12" t="s">
@@ -37614,10 +37614,10 @@
     </row>
     <row r="8675" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8675" s="4"/>
-      <c r="B8675" s="36" t="s">
+      <c r="B8675" s="38" t="s">
         <v>380</v>
       </c>
-      <c r="C8675" s="37"/>
+      <c r="C8675" s="39"/>
     </row>
     <row r="8676" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8676" s="12" t="s">
@@ -37869,14 +37869,14 @@
         <v>3.1</v>
       </c>
       <c r="B8741" s="9"/>
-      <c r="C8741" s="39" t="s">
+      <c r="C8741" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="8742" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8742" s="8"/>
       <c r="B8742" s="9"/>
-      <c r="C8742" s="39"/>
+      <c r="C8742" s="36"/>
     </row>
     <row r="8743" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8743" s="15">
@@ -38009,14 +38009,14 @@
         <v>3.1</v>
       </c>
       <c r="B8800" s="9"/>
-      <c r="C8800" s="39" t="s">
+      <c r="C8800" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="8801" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8801" s="8"/>
       <c r="B8801" s="9"/>
-      <c r="C8801" s="39"/>
+      <c r="C8801" s="36"/>
     </row>
     <row r="8802" spans="1:3" s="28" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8802" s="15">
@@ -38149,14 +38149,14 @@
         <v>3.1</v>
       </c>
       <c r="B8859" s="9"/>
-      <c r="C8859" s="39" t="s">
+      <c r="C8859" s="36" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="8860" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8860" s="8"/>
       <c r="B8860" s="9"/>
-      <c r="C8860" s="39"/>
+      <c r="C8860" s="36"/>
     </row>
     <row r="8861" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8861" s="15">
@@ -38221,10 +38221,10 @@
     </row>
     <row r="8911" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8911" s="4"/>
-      <c r="B8911" s="36" t="s">
+      <c r="B8911" s="38" t="s">
         <v>386</v>
       </c>
-      <c r="C8911" s="37"/>
+      <c r="C8911" s="39"/>
     </row>
     <row r="8912" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8912" s="12" t="s">
@@ -38315,7 +38315,7 @@
       <c r="A8921" s="8">
         <v>4.2</v>
       </c>
-      <c r="B8921" s="38" t="s">
+      <c r="B8921" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C8921" s="14" t="s">
@@ -38324,12 +38324,12 @@
     </row>
     <row r="8922" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8922" s="8"/>
-      <c r="B8922" s="38"/>
+      <c r="B8922" s="37"/>
       <c r="C8922" s="14"/>
     </row>
     <row r="8923" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8923" s="8"/>
-      <c r="B8923" s="38"/>
+      <c r="B8923" s="37"/>
       <c r="C8923" s="14"/>
     </row>
     <row r="8924" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -38343,7 +38343,7 @@
       <c r="A8925" s="8">
         <v>5.2</v>
       </c>
-      <c r="B8925" s="38" t="s">
+      <c r="B8925" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C8925" s="14" t="s">
@@ -38352,12 +38352,12 @@
     </row>
     <row r="8926" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8926" s="8"/>
-      <c r="B8926" s="38"/>
+      <c r="B8926" s="37"/>
       <c r="C8926" s="14"/>
     </row>
     <row r="8927" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8927" s="8"/>
-      <c r="B8927" s="38"/>
+      <c r="B8927" s="37"/>
       <c r="C8927" s="14"/>
     </row>
     <row r="8928" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -39529,10 +39529,10 @@
     </row>
     <row r="9501" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9501" s="4"/>
-      <c r="B9501" s="36" t="s">
+      <c r="B9501" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C9501" s="37"/>
+      <c r="C9501" s="39"/>
     </row>
     <row r="9502" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9502" s="12" t="s">
@@ -39653,7 +39653,7 @@
       <c r="A9515" s="8">
         <v>5.2</v>
       </c>
-      <c r="B9515" s="38" t="s">
+      <c r="B9515" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C9515" s="10" t="s">
@@ -39662,12 +39662,12 @@
     </row>
     <row r="9516" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9516" s="8"/>
-      <c r="B9516" s="38"/>
+      <c r="B9516" s="37"/>
       <c r="C9516" s="10"/>
     </row>
     <row r="9517" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9517" s="8"/>
-      <c r="B9517" s="38"/>
+      <c r="B9517" s="37"/>
       <c r="C9517" s="10"/>
     </row>
     <row r="9518" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -41436,14 +41436,14 @@
       <c r="B10390" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C10390" s="39" t="s">
+      <c r="C10390" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="10391" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10391" s="8"/>
       <c r="B10391" s="9"/>
-      <c r="C10391" s="39"/>
+      <c r="C10391" s="36"/>
     </row>
     <row r="10392" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10392" s="8">
@@ -41519,10 +41519,10 @@
     </row>
     <row r="10445" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10445" s="4"/>
-      <c r="B10445" s="36" t="s">
+      <c r="B10445" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C10445" s="37"/>
+      <c r="C10445" s="39"/>
     </row>
     <row r="10446" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10446" s="12" t="s">
@@ -41881,10 +41881,10 @@
     </row>
     <row r="10563" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10563" s="4"/>
-      <c r="B10563" s="36" t="s">
+      <c r="B10563" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="C10563" s="37"/>
+      <c r="C10563" s="39"/>
     </row>
     <row r="10564" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10564" s="12" t="s">
@@ -42136,14 +42136,14 @@
         <v>3.1</v>
       </c>
       <c r="B10629" s="9"/>
-      <c r="C10629" s="39" t="s">
+      <c r="C10629" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="10630" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10630" s="8"/>
       <c r="B10630" s="9"/>
-      <c r="C10630" s="39"/>
+      <c r="C10630" s="36"/>
     </row>
     <row r="10631" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10631" s="15">
@@ -42278,14 +42278,14 @@
         <v>3.1</v>
       </c>
       <c r="B10688" s="9"/>
-      <c r="C10688" s="39" t="s">
+      <c r="C10688" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="10689" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10689" s="8"/>
       <c r="B10689" s="9"/>
-      <c r="C10689" s="39"/>
+      <c r="C10689" s="36"/>
     </row>
     <row r="10690" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10690" s="15">
@@ -42420,14 +42420,14 @@
         <v>3.1</v>
       </c>
       <c r="B10747" s="9"/>
-      <c r="C10747" s="39" t="s">
+      <c r="C10747" s="36" t="s">
         <v>384</v>
       </c>
     </row>
     <row r="10748" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10748" s="8"/>
       <c r="B10748" s="9"/>
-      <c r="C10748" s="39"/>
+      <c r="C10748" s="36"/>
     </row>
     <row r="10749" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10749" s="15">
@@ -42494,10 +42494,10 @@
     </row>
     <row r="10799" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10799" s="4"/>
-      <c r="B10799" s="36" t="s">
+      <c r="B10799" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C10799" s="37"/>
+      <c r="C10799" s="39"/>
     </row>
     <row r="10800" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10800" s="12" t="s">
@@ -42588,7 +42588,7 @@
       <c r="A10809" s="8">
         <v>4.2</v>
       </c>
-      <c r="B10809" s="38" t="s">
+      <c r="B10809" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C10809" s="10" t="s">
@@ -42597,12 +42597,12 @@
     </row>
     <row r="10810" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10810" s="8"/>
-      <c r="B10810" s="38"/>
+      <c r="B10810" s="37"/>
       <c r="C10810" s="10"/>
     </row>
     <row r="10811" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10811" s="8"/>
-      <c r="B10811" s="38"/>
+      <c r="B10811" s="37"/>
       <c r="C10811" s="10"/>
     </row>
     <row r="10812" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -42616,7 +42616,7 @@
       <c r="A10813" s="8">
         <v>5.2</v>
       </c>
-      <c r="B10813" s="38" t="s">
+      <c r="B10813" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C10813" s="10" t="s">
@@ -42625,12 +42625,12 @@
     </row>
     <row r="10814" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10814" s="8"/>
-      <c r="B10814" s="38"/>
+      <c r="B10814" s="37"/>
       <c r="C10814" s="10"/>
     </row>
     <row r="10815" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10815" s="8"/>
-      <c r="B10815" s="38"/>
+      <c r="B10815" s="37"/>
       <c r="C10815" s="10"/>
     </row>
     <row r="10816" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -43857,14 +43857,14 @@
         <v>2.1</v>
       </c>
       <c r="B11335" s="9"/>
-      <c r="C11335" s="39" t="s">
+      <c r="C11335" s="36" t="s">
         <v>450</v>
       </c>
     </row>
     <row r="11336" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11336" s="8"/>
       <c r="B11336" s="9"/>
-      <c r="C11336" s="39"/>
+      <c r="C11336" s="36"/>
     </row>
     <row r="11337" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11337" s="8">
@@ -43897,10 +43897,10 @@
     </row>
     <row r="11389" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11389" s="4"/>
-      <c r="B11389" s="36" t="s">
+      <c r="B11389" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C11389" s="37"/>
+      <c r="C11389" s="39"/>
     </row>
     <row r="11390" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11390" s="12" t="s">
@@ -44021,7 +44021,7 @@
       <c r="A11403" s="8">
         <v>5.2</v>
       </c>
-      <c r="B11403" s="38" t="s">
+      <c r="B11403" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C11403" s="10" t="s">
@@ -44030,12 +44030,12 @@
     </row>
     <row r="11404" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11404" s="8"/>
-      <c r="B11404" s="38"/>
+      <c r="B11404" s="37"/>
       <c r="C11404" s="10"/>
     </row>
     <row r="11405" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11405" s="8"/>
-      <c r="B11405" s="38"/>
+      <c r="B11405" s="37"/>
       <c r="C11405" s="10"/>
     </row>
     <row r="11406" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -44061,14 +44061,14 @@
         <v>7.1</v>
       </c>
       <c r="B11408" s="9"/>
-      <c r="C11408" s="39" t="s">
+      <c r="C11408" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="11409" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11409" s="8"/>
       <c r="B11409" s="9"/>
-      <c r="C11409" s="39"/>
+      <c r="C11409" s="36"/>
     </row>
     <row r="11410" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11410" s="8">
@@ -44295,14 +44295,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B11516" s="9"/>
-      <c r="C11516" s="39" t="s">
+      <c r="C11516" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="11517" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11517" s="8"/>
       <c r="B11517" s="9"/>
-      <c r="C11517" s="39"/>
+      <c r="C11517" s="36"/>
     </row>
     <row r="11518" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11518" s="8">
@@ -44423,14 +44423,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B11575" s="9"/>
-      <c r="C11575" s="39" t="s">
+      <c r="C11575" s="36" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="11576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11576" s="8"/>
       <c r="B11576" s="9"/>
-      <c r="C11576" s="39"/>
+      <c r="C11576" s="36"/>
     </row>
     <row r="11577" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11577" s="8">
@@ -44551,14 +44551,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B11634" s="9"/>
-      <c r="C11634" s="39" t="s">
+      <c r="C11634" s="36" t="s">
         <v>459</v>
       </c>
     </row>
     <row r="11635" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11635" s="8"/>
       <c r="B11635" s="9"/>
-      <c r="C11635" s="39"/>
+      <c r="C11635" s="36"/>
     </row>
     <row r="11636" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11636" s="8">
@@ -44892,14 +44892,14 @@
         <v>7.1</v>
       </c>
       <c r="B11758" s="9"/>
-      <c r="C11758" s="39" t="s">
+      <c r="C11758" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="11759" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11759" s="8"/>
       <c r="B11759" s="9"/>
-      <c r="C11759" s="39"/>
+      <c r="C11759" s="36"/>
     </row>
     <row r="11760" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11760" s="8">
@@ -45071,14 +45071,14 @@
         <v>2.1</v>
       </c>
       <c r="B11866" s="9"/>
-      <c r="C11866" s="39" t="s">
+      <c r="C11866" s="36" t="s">
         <v>465</v>
       </c>
     </row>
     <row r="11867" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11867" s="8"/>
       <c r="B11867" s="9"/>
-      <c r="C11867" s="39"/>
+      <c r="C11867" s="36"/>
     </row>
     <row r="11868" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11868" s="8">
@@ -45380,14 +45380,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B12047" s="9"/>
-      <c r="C12047" s="39" t="s">
+      <c r="C12047" s="36" t="s">
         <v>457</v>
       </c>
     </row>
     <row r="12048" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12048" s="8"/>
       <c r="B12048" s="9"/>
-      <c r="C12048" s="39"/>
+      <c r="C12048" s="36"/>
     </row>
     <row r="12049" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12049" s="8">
@@ -45512,14 +45512,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B12106" s="9"/>
-      <c r="C12106" s="39" t="s">
+      <c r="C12106" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12107" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12107" s="8"/>
       <c r="B12107" s="9"/>
-      <c r="C12107" s="39"/>
+      <c r="C12107" s="36"/>
     </row>
     <row r="12108" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12108" s="8">
@@ -45552,10 +45552,10 @@
     </row>
     <row r="12156" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12156" s="4"/>
-      <c r="B12156" s="36" t="s">
+      <c r="B12156" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C12156" s="37"/>
+      <c r="C12156" s="39"/>
     </row>
     <row r="12157" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12157" s="12" t="s">
@@ -45827,14 +45827,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B12226" s="9"/>
-      <c r="C12226" s="39" t="s">
+      <c r="C12226" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12227" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12227" s="8"/>
       <c r="B12227" s="9"/>
-      <c r="C12227" s="39"/>
+      <c r="C12227" s="36"/>
     </row>
     <row r="12228" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12228" s="8">
@@ -45910,14 +45910,14 @@
       <c r="B12278" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C12278" s="39" t="s">
+      <c r="C12278" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="12279" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12279" s="8"/>
       <c r="B12279" s="9"/>
-      <c r="C12279" s="39"/>
+      <c r="C12279" s="36"/>
     </row>
     <row r="12280" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12280" s="8">
@@ -45993,10 +45993,10 @@
     </row>
     <row r="12333" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12333" s="4"/>
-      <c r="B12333" s="36" t="s">
+      <c r="B12333" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C12333" s="37"/>
+      <c r="C12333" s="39"/>
     </row>
     <row r="12334" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12334" s="12" t="s">
@@ -46161,14 +46161,14 @@
         <v>7.1</v>
       </c>
       <c r="B12352" s="9"/>
-      <c r="C12352" s="39" t="s">
+      <c r="C12352" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12353" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12353" s="8"/>
       <c r="B12353" s="9"/>
-      <c r="C12353" s="39"/>
+      <c r="C12353" s="36"/>
     </row>
     <row r="12354" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12354" s="8">
@@ -46325,14 +46325,14 @@
         <v>6.1</v>
       </c>
       <c r="B12405" s="9"/>
-      <c r="C12405" s="39" t="s">
+      <c r="C12405" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12406" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12406" s="8"/>
       <c r="B12406" s="9"/>
-      <c r="C12406" s="39"/>
+      <c r="C12406" s="36"/>
     </row>
     <row r="12407" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12407" s="8">
@@ -46365,10 +46365,10 @@
     </row>
     <row r="12451" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12451" s="4"/>
-      <c r="B12451" s="36" t="s">
+      <c r="B12451" s="38" t="s">
         <v>99</v>
       </c>
-      <c r="C12451" s="37"/>
+      <c r="C12451" s="39"/>
     </row>
     <row r="12452" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12452" s="12" t="s">
@@ -46517,14 +46517,14 @@
         <v>7.1</v>
       </c>
       <c r="B12468" s="9"/>
-      <c r="C12468" s="39" t="s">
+      <c r="C12468" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12469" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12469" s="8"/>
       <c r="B12469" s="9"/>
-      <c r="C12469" s="39"/>
+      <c r="C12469" s="36"/>
     </row>
     <row r="12470" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12470" s="8">
@@ -46557,10 +46557,10 @@
     </row>
     <row r="12510" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12510" s="4"/>
-      <c r="B12510" s="36" t="s">
+      <c r="B12510" s="38" t="s">
         <v>505</v>
       </c>
-      <c r="C12510" s="37"/>
+      <c r="C12510" s="39"/>
     </row>
     <row r="12511" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12511" s="12" t="s">
@@ -46651,7 +46651,7 @@
       <c r="A12520" s="8">
         <v>4.2</v>
       </c>
-      <c r="B12520" s="38" t="s">
+      <c r="B12520" s="37" t="s">
         <v>506</v>
       </c>
       <c r="C12520" s="10" t="s">
@@ -46660,12 +46660,12 @@
     </row>
     <row r="12521" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12521" s="8"/>
-      <c r="B12521" s="38"/>
+      <c r="B12521" s="37"/>
       <c r="C12521" s="10"/>
     </row>
     <row r="12522" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12522" s="8"/>
-      <c r="B12522" s="38"/>
+      <c r="B12522" s="37"/>
       <c r="C12522" s="10"/>
     </row>
     <row r="12523" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -46812,14 +46812,14 @@
         <v>3.1</v>
       </c>
       <c r="B12576" s="9"/>
-      <c r="C12576" s="39" t="s">
+      <c r="C12576" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="12577" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12577" s="8"/>
       <c r="B12577" s="9"/>
-      <c r="C12577" s="39"/>
+      <c r="C12577" s="36"/>
     </row>
     <row r="12578" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12578" s="8">
@@ -46851,14 +46851,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B12581" s="27"/>
-      <c r="C12581" s="39" t="s">
+      <c r="C12581" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12582" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12582" s="8"/>
       <c r="B12582" s="27"/>
-      <c r="C12582" s="39"/>
+      <c r="C12582" s="36"/>
     </row>
     <row r="12583" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12583" s="8">
@@ -46891,10 +46891,10 @@
     </row>
     <row r="12628" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12628" s="4"/>
-      <c r="B12628" s="36" t="s">
+      <c r="B12628" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="C12628" s="37"/>
+      <c r="C12628" s="39"/>
     </row>
     <row r="12629" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12629" s="12" t="s">
@@ -46959,28 +46959,28 @@
         <v>3.1</v>
       </c>
       <c r="B12635" s="9"/>
-      <c r="C12635" s="39" t="s">
+      <c r="C12635" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="12636" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12636" s="8"/>
       <c r="B12636" s="9"/>
-      <c r="C12636" s="39"/>
+      <c r="C12636" s="36"/>
     </row>
     <row r="12637" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12637" s="8">
+      <c r="A12637" s="15">
         <v>3.2</v>
       </c>
-      <c r="B12637" s="9"/>
-      <c r="C12637" s="10"/>
+      <c r="B12637" s="16"/>
+      <c r="C12637" s="23"/>
     </row>
     <row r="12638" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12638" s="8">
+      <c r="A12638" s="15">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B12638" s="9"/>
-      <c r="C12638" s="10"/>
+      <c r="B12638" s="16"/>
+      <c r="C12638" s="23"/>
     </row>
     <row r="12639" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12639" s="8">
@@ -47069,10 +47069,10 @@
     </row>
     <row r="12687" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12687" s="4"/>
-      <c r="B12687" s="36" t="s">
+      <c r="B12687" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C12687" s="37"/>
+      <c r="C12687" s="39"/>
     </row>
     <row r="12688" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12688" s="12" t="s">
@@ -47163,7 +47163,7 @@
       <c r="A12697" s="8">
         <v>4.2</v>
       </c>
-      <c r="B12697" s="38" t="s">
+      <c r="B12697" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C12697" s="10" t="s">
@@ -47172,12 +47172,12 @@
     </row>
     <row r="12698" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12698" s="8"/>
-      <c r="B12698" s="38"/>
+      <c r="B12698" s="37"/>
       <c r="C12698" s="10"/>
     </row>
     <row r="12699" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12699" s="8"/>
-      <c r="B12699" s="38"/>
+      <c r="B12699" s="37"/>
       <c r="C12699" s="10"/>
     </row>
     <row r="12700" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -47191,7 +47191,7 @@
       <c r="A12701" s="8">
         <v>5.2</v>
       </c>
-      <c r="B12701" s="38" t="s">
+      <c r="B12701" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C12701" s="10" t="s">
@@ -47200,12 +47200,12 @@
     </row>
     <row r="12702" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12702" s="8"/>
-      <c r="B12702" s="38"/>
+      <c r="B12702" s="37"/>
       <c r="C12702" s="10"/>
     </row>
     <row r="12703" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12703" s="8"/>
-      <c r="B12703" s="38"/>
+      <c r="B12703" s="37"/>
       <c r="C12703" s="10"/>
     </row>
     <row r="12704" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -47247,14 +47247,14 @@
         <v>7.1</v>
       </c>
       <c r="B12708" s="9"/>
-      <c r="C12708" s="39" t="s">
+      <c r="C12708" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12709" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12709" s="8"/>
       <c r="B12709" s="9"/>
-      <c r="C12709" s="39"/>
+      <c r="C12709" s="36"/>
     </row>
     <row r="12710" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12710" s="8">
@@ -47508,14 +47508,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B12820" s="27"/>
-      <c r="C12820" s="39" t="s">
+      <c r="C12820" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="12821" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12821" s="8"/>
       <c r="B12821" s="27"/>
-      <c r="C12821" s="39"/>
+      <c r="C12821" s="36"/>
     </row>
     <row r="12822" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12822" s="8">
@@ -47742,10 +47742,10 @@
     </row>
     <row r="12982" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12982" s="4"/>
-      <c r="B12982" s="36" t="s">
+      <c r="B12982" s="38" t="s">
         <v>520</v>
       </c>
-      <c r="C12982" s="37"/>
+      <c r="C12982" s="39"/>
     </row>
     <row r="12983" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12983" s="12" t="s">
@@ -47858,7 +47858,7 @@
       <c r="A12994" s="18">
         <v>5.2</v>
       </c>
-      <c r="B12994" s="38" t="s">
+      <c r="B12994" s="37" t="s">
         <v>521</v>
       </c>
       <c r="C12994" s="10" t="s">
@@ -47867,12 +47867,12 @@
     </row>
     <row r="12995" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12995" s="18"/>
-      <c r="B12995" s="38"/>
+      <c r="B12995" s="37"/>
       <c r="C12995" s="10"/>
     </row>
     <row r="12996" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12996" s="18"/>
-      <c r="B12996" s="38"/>
+      <c r="B12996" s="37"/>
       <c r="C12996" s="10"/>
     </row>
     <row r="12997" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -48049,14 +48049,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B13056" s="9"/>
-      <c r="C13056" s="39" t="s">
+      <c r="C13056" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="13057" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13057" s="8"/>
       <c r="B13057" s="9"/>
-      <c r="C13057" s="39"/>
+      <c r="C13057" s="36"/>
     </row>
     <row r="13058" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13058" s="8">
@@ -48089,10 +48089,10 @@
     </row>
     <row r="13100" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13100" s="4"/>
-      <c r="B13100" s="36" t="s">
+      <c r="B13100" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="C13100" s="37"/>
+      <c r="C13100" s="39"/>
     </row>
     <row r="13101" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13101" s="12" t="s">
@@ -48406,14 +48406,14 @@
         <v>5.0999999999999996</v>
       </c>
       <c r="B13172" s="9"/>
-      <c r="C13172" s="39" t="s">
+      <c r="C13172" s="36" t="s">
         <v>452</v>
       </c>
     </row>
     <row r="13173" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13173" s="8"/>
       <c r="B13173" s="9"/>
-      <c r="C13173" s="39"/>
+      <c r="C13173" s="36"/>
     </row>
     <row r="13174" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13174" s="8">
@@ -48498,14 +48498,14 @@
         <v>2.1</v>
       </c>
       <c r="B13223" s="9"/>
-      <c r="C13223" s="39" t="s">
+      <c r="C13223" s="36" t="s">
         <v>527</v>
       </c>
     </row>
     <row r="13224" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13224" s="8"/>
       <c r="B13224" s="9"/>
-      <c r="C13224" s="39"/>
+      <c r="C13224" s="36"/>
     </row>
     <row r="13225" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13225" s="8">
@@ -48538,10 +48538,10 @@
     </row>
     <row r="13277" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13277" s="4"/>
-      <c r="B13277" s="36" t="s">
+      <c r="B13277" s="38" t="s">
         <v>52</v>
       </c>
-      <c r="C13277" s="37"/>
+      <c r="C13277" s="39"/>
     </row>
     <row r="13278" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13278" s="12" t="s">
@@ -48662,7 +48662,7 @@
       <c r="A13291" s="8">
         <v>5.2</v>
       </c>
-      <c r="B13291" s="38" t="s">
+      <c r="B13291" s="37" t="s">
         <v>584</v>
       </c>
       <c r="C13291" s="10" t="s">
@@ -48671,12 +48671,12 @@
     </row>
     <row r="13292" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13292" s="8"/>
-      <c r="B13292" s="38"/>
+      <c r="B13292" s="37"/>
       <c r="C13292" s="10"/>
     </row>
     <row r="13293" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13293" s="8"/>
-      <c r="B13293" s="38"/>
+      <c r="B13293" s="37"/>
       <c r="C13293" s="10"/>
     </row>
     <row r="13294" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -48687,7 +48687,7 @@
       <c r="C13294" s="10"/>
     </row>
     <row r="13295" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13295" s="8">
+      <c r="A13295" s="18">
         <v>6.2</v>
       </c>
       <c r="B13295" s="9" t="s">
@@ -49012,7 +49012,7 @@
       <c r="C13402" s="10"/>
     </row>
     <row r="13403" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13403" s="8">
+      <c r="A13403" s="18">
         <v>3.2</v>
       </c>
       <c r="B13403" s="9" t="s">
@@ -49248,14 +49248,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B13463" s="9"/>
-      <c r="C13463" s="39" t="s">
+      <c r="C13463" s="36" t="s">
         <v>543</v>
       </c>
     </row>
     <row r="13464" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13464" s="8"/>
       <c r="B13464" s="9"/>
-      <c r="C13464" s="39"/>
+      <c r="C13464" s="36"/>
     </row>
     <row r="13465" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13465" s="8">
@@ -49668,10 +49668,10 @@
     </row>
     <row r="13631" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13631" s="4"/>
-      <c r="B13631" s="36" t="s">
+      <c r="B13631" s="38" t="s">
         <v>71</v>
       </c>
-      <c r="C13631" s="37"/>
+      <c r="C13631" s="39"/>
     </row>
     <row r="13632" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13632" s="12" t="s">
@@ -50489,14 +50489,14 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="B13935" s="9"/>
-      <c r="C13935" s="39" t="s">
+      <c r="C13935" s="36" t="s">
         <v>543</v>
       </c>
     </row>
     <row r="13936" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13936" s="8"/>
       <c r="B13936" s="9"/>
-      <c r="C13936" s="39"/>
+      <c r="C13936" s="36"/>
     </row>
     <row r="13937" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13937" s="8">
@@ -50754,10 +50754,10 @@
     </row>
     <row r="14044" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14044" s="4"/>
-      <c r="B14044" s="36" t="s">
+      <c r="B14044" s="38" t="s">
         <v>28</v>
       </c>
-      <c r="C14044" s="37"/>
+      <c r="C14044" s="39"/>
     </row>
     <row r="14045" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14045" s="12" t="s">
@@ -51205,14 +51205,14 @@
       <c r="B14166" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="C14166" s="39" t="s">
+      <c r="C14166" s="36" t="s">
         <v>178</v>
       </c>
     </row>
     <row r="14167" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14167" s="8"/>
       <c r="B14167" s="9"/>
-      <c r="C14167" s="39"/>
+      <c r="C14167" s="36"/>
     </row>
     <row r="14168" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14168" s="8">
@@ -51288,10 +51288,10 @@
     </row>
     <row r="14221" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14221" s="4"/>
-      <c r="B14221" s="36" t="s">
+      <c r="B14221" s="38" t="s">
         <v>94</v>
       </c>
-      <c r="C14221" s="37"/>
+      <c r="C14221" s="39"/>
     </row>
     <row r="14222" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14222" s="12" t="s">
@@ -52276,10 +52276,10 @@
     </row>
     <row r="14457" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14457" s="4"/>
-      <c r="B14457" s="36" t="s">
+      <c r="B14457" s="38" t="s">
         <v>105</v>
       </c>
-      <c r="C14457" s="37"/>
+      <c r="C14457" s="39"/>
     </row>
     <row r="14458" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14458" s="12" t="s">
@@ -52344,14 +52344,14 @@
         <v>3.1</v>
       </c>
       <c r="B14464" s="9"/>
-      <c r="C14464" s="39" t="s">
+      <c r="C14464" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="14465" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14465" s="8"/>
       <c r="B14465" s="9"/>
-      <c r="C14465" s="39"/>
+      <c r="C14465" s="36"/>
     </row>
     <row r="14466" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14466" s="15">
@@ -52516,10 +52516,10 @@
     </row>
     <row r="14516" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14516" s="4"/>
-      <c r="B14516" s="36" t="s">
+      <c r="B14516" s="38" t="s">
         <v>196</v>
       </c>
-      <c r="C14516" s="37"/>
+      <c r="C14516" s="39"/>
     </row>
     <row r="14517" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14517" s="12" t="s">
@@ -52584,28 +52584,28 @@
         <v>3.1</v>
       </c>
       <c r="B14523" s="9"/>
-      <c r="C14523" s="39" t="s">
+      <c r="C14523" s="36" t="s">
         <v>155</v>
       </c>
     </row>
     <row r="14524" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14524" s="8"/>
       <c r="B14524" s="9"/>
-      <c r="C14524" s="39"/>
+      <c r="C14524" s="36"/>
     </row>
     <row r="14525" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14525" s="8">
+      <c r="A14525" s="15">
         <v>3.2</v>
       </c>
-      <c r="B14525" s="9"/>
-      <c r="C14525" s="10"/>
+      <c r="B14525" s="16"/>
+      <c r="C14525" s="23"/>
     </row>
     <row r="14526" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14526" s="8">
+      <c r="A14526" s="15">
         <v>4.0999999999999996</v>
       </c>
-      <c r="B14526" s="9"/>
-      <c r="C14526" s="10"/>
+      <c r="B14526" s="16"/>
+      <c r="C14526" s="23"/>
     </row>
     <row r="14527" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14527" s="8">
@@ -52694,10 +52694,10 @@
     </row>
     <row r="14575" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14575" s="4"/>
-      <c r="B14575" s="36" t="s">
+      <c r="B14575" s="38" t="s">
         <v>111</v>
       </c>
-      <c r="C14575" s="37"/>
+      <c r="C14575" s="39"/>
     </row>
     <row r="14576" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14576" s="12" t="s">
@@ -52788,7 +52788,7 @@
       <c r="A14585" s="8">
         <v>4.2</v>
       </c>
-      <c r="B14585" s="38" t="s">
+      <c r="B14585" s="37" t="s">
         <v>156</v>
       </c>
       <c r="C14585" s="10" t="s">
@@ -52797,12 +52797,12 @@
     </row>
     <row r="14586" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14586" s="8"/>
-      <c r="B14586" s="38"/>
+      <c r="B14586" s="37"/>
       <c r="C14586" s="10"/>
     </row>
     <row r="14587" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14587" s="8"/>
-      <c r="B14587" s="38"/>
+      <c r="B14587" s="37"/>
       <c r="C14587" s="10"/>
     </row>
     <row r="14588" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -52816,7 +52816,7 @@
       <c r="A14589" s="8">
         <v>5.2</v>
       </c>
-      <c r="B14589" s="38" t="s">
+      <c r="B14589" s="37" t="s">
         <v>157</v>
       </c>
       <c r="C14589" s="10" t="s">
@@ -52825,12 +52825,12 @@
     </row>
     <row r="14590" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14590" s="8"/>
-      <c r="B14590" s="38"/>
+      <c r="B14590" s="37"/>
       <c r="C14590" s="10"/>
     </row>
     <row r="14591" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14591" s="8"/>
-      <c r="B14591" s="38"/>
+      <c r="B14591" s="37"/>
       <c r="C14591" s="10"/>
     </row>
     <row r="14592" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -53528,14 +53528,14 @@
         <v>2.1</v>
       </c>
       <c r="B14816" s="27"/>
-      <c r="C14816" s="38" t="s">
+      <c r="C14816" s="37" t="s">
         <v>575</v>
       </c>
     </row>
     <row r="14817" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14817" s="8"/>
       <c r="B14817" s="27"/>
-      <c r="C14817" s="38"/>
+      <c r="C14817" s="37"/>
     </row>
     <row r="14818" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14818" s="8">
@@ -53568,10 +53568,10 @@
     </row>
     <row r="14870" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14870" s="4"/>
-      <c r="B14870" s="36" t="s">
+      <c r="B14870" s="38" t="s">
         <v>577</v>
       </c>
-      <c r="C14870" s="37"/>
+      <c r="C14870" s="39"/>
     </row>
     <row r="14871" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14871" s="12" t="s">
@@ -54039,10 +54039,10 @@
     </row>
     <row r="14988" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14988" s="4"/>
-      <c r="B14988" s="36" t="s">
+      <c r="B14988" s="38" t="s">
         <v>124</v>
       </c>
-      <c r="C14988" s="37"/>
+      <c r="C14988" s="39"/>
     </row>
     <row r="14989" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14989" s="12" t="s">
@@ -54230,10 +54230,10 @@
     </row>
     <row r="15047" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15047" s="4"/>
-      <c r="B15047" s="36" t="s">
+      <c r="B15047" s="38" t="s">
         <v>128</v>
       </c>
-      <c r="C15047" s="37"/>
+      <c r="C15047" s="39"/>
     </row>
     <row r="15048" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15048" s="12" t="s">
@@ -54478,117 +54478,54 @@
     </row>
   </sheetData>
   <mergeCells count="182">
-    <mergeCell ref="C8741:C8742"/>
-    <mergeCell ref="B7627:B7629"/>
-    <mergeCell ref="C8502:C8503"/>
-    <mergeCell ref="B8557:C8557"/>
-    <mergeCell ref="B8675:C8675"/>
-    <mergeCell ref="B7613:C7613"/>
-    <mergeCell ref="B5784:C5784"/>
-    <mergeCell ref="B7672:C7672"/>
-    <mergeCell ref="B6020:C6020"/>
-    <mergeCell ref="C6853:C6854"/>
-    <mergeCell ref="C6912:C6913"/>
-    <mergeCell ref="C6971:C6972"/>
-    <mergeCell ref="B6964:C6964"/>
-    <mergeCell ref="C7451:C7452"/>
-    <mergeCell ref="B7436:C7436"/>
-    <mergeCell ref="C7558:C7559"/>
-    <mergeCell ref="B7209:B7211"/>
-    <mergeCell ref="B7318:C7318"/>
-    <mergeCell ref="C6978:C6979"/>
-    <mergeCell ref="B7023:C7023"/>
-    <mergeCell ref="B7033:B7035"/>
-    <mergeCell ref="B7037:B7039"/>
-    <mergeCell ref="B5607:C5607"/>
-    <mergeCell ref="B5430:C5430"/>
-    <mergeCell ref="B5489:C5489"/>
-    <mergeCell ref="B5548:C5548"/>
-    <mergeCell ref="C5563:C5564"/>
-    <mergeCell ref="B6669:C6669"/>
-    <mergeCell ref="B6787:C6787"/>
-    <mergeCell ref="C6031:C6032"/>
-    <mergeCell ref="B6492:C6492"/>
-    <mergeCell ref="C6503:C6504"/>
-    <mergeCell ref="C6614:C6615"/>
-    <mergeCell ref="B5739:B5741"/>
-    <mergeCell ref="B5725:C5725"/>
-    <mergeCell ref="C5024:C5025"/>
-    <mergeCell ref="B4781:C4781"/>
-    <mergeCell ref="C4969:C4970"/>
-    <mergeCell ref="B4899:C4899"/>
-    <mergeCell ref="C4615:C4616"/>
-    <mergeCell ref="B5135:C5135"/>
-    <mergeCell ref="B5145:B5147"/>
-    <mergeCell ref="B5149:B5151"/>
-    <mergeCell ref="B5076:C5076"/>
-    <mergeCell ref="C5083:C5084"/>
-    <mergeCell ref="C5090:C5091"/>
-    <mergeCell ref="B3365:C3365"/>
-    <mergeCell ref="C3675:C3676"/>
-    <mergeCell ref="B3257:B3259"/>
-    <mergeCell ref="B3261:B3263"/>
-    <mergeCell ref="B3247:C3247"/>
-    <mergeCell ref="B4604:C4604"/>
-    <mergeCell ref="B4663:C4663"/>
-    <mergeCell ref="C4726:C4727"/>
-    <mergeCell ref="B3660:C3660"/>
-    <mergeCell ref="B3837:C3837"/>
-    <mergeCell ref="B3896:C3896"/>
-    <mergeCell ref="C4143:C4144"/>
-    <mergeCell ref="B4191:C4191"/>
-    <mergeCell ref="B4014:C4014"/>
-    <mergeCell ref="C4025:C4026"/>
-    <mergeCell ref="B4132:C4132"/>
-    <mergeCell ref="B3851:B3853"/>
-    <mergeCell ref="B2775:C2775"/>
-    <mergeCell ref="C2838:C2839"/>
-    <mergeCell ref="B2893:C2893"/>
-    <mergeCell ref="B2657:C2657"/>
-    <mergeCell ref="B2716:C2716"/>
-    <mergeCell ref="C2727:C2728"/>
-    <mergeCell ref="C3202:C3203"/>
-    <mergeCell ref="B3188:C3188"/>
-    <mergeCell ref="C3077:C3078"/>
-    <mergeCell ref="C3136:C3137"/>
-    <mergeCell ref="C3195:C3196"/>
-    <mergeCell ref="B3011:C3011"/>
-    <mergeCell ref="C2255:C2256"/>
-    <mergeCell ref="B2244:C2244"/>
-    <mergeCell ref="B1949:C1949"/>
-    <mergeCell ref="B1890:C1890"/>
-    <mergeCell ref="B1831:C1831"/>
-    <mergeCell ref="B1772:C1772"/>
-    <mergeCell ref="B1713:C1713"/>
-    <mergeCell ref="C1787:C1788"/>
-    <mergeCell ref="B1654:C1654"/>
-    <mergeCell ref="B1963:B1965"/>
-    <mergeCell ref="B1477:C1477"/>
-    <mergeCell ref="B1359:C1359"/>
-    <mergeCell ref="B1300:C1300"/>
-    <mergeCell ref="B887:C887"/>
-    <mergeCell ref="C950:C951"/>
-    <mergeCell ref="B1064:C1064"/>
-    <mergeCell ref="C1248:C1249"/>
-    <mergeCell ref="C367:C368"/>
-    <mergeCell ref="B415:C415"/>
-    <mergeCell ref="B710:C710"/>
-    <mergeCell ref="B828:C828"/>
-    <mergeCell ref="C839:C840"/>
-    <mergeCell ref="C1307:C1308"/>
-    <mergeCell ref="C1314:C1315"/>
-    <mergeCell ref="B1369:B1371"/>
-    <mergeCell ref="B1373:B1375"/>
-    <mergeCell ref="B1123:C1123"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B1182:C1182"/>
-    <mergeCell ref="B1005:C1005"/>
-    <mergeCell ref="A145:C145"/>
-    <mergeCell ref="A24:C27"/>
-    <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="B179:C179"/>
-    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B14988:C14988"/>
+    <mergeCell ref="B15047:C15047"/>
+    <mergeCell ref="C14816:C14817"/>
+    <mergeCell ref="B14870:C14870"/>
+    <mergeCell ref="C14523:C14524"/>
+    <mergeCell ref="B14516:C14516"/>
+    <mergeCell ref="B14457:C14457"/>
+    <mergeCell ref="B14575:C14575"/>
+    <mergeCell ref="B14585:B14587"/>
+    <mergeCell ref="B14589:B14591"/>
+    <mergeCell ref="B13631:C13631"/>
+    <mergeCell ref="C13935:C13936"/>
+    <mergeCell ref="B14044:C14044"/>
+    <mergeCell ref="C14166:C14167"/>
+    <mergeCell ref="B14221:C14221"/>
+    <mergeCell ref="C14464:C14465"/>
+    <mergeCell ref="C13223:C13224"/>
+    <mergeCell ref="B13277:C13277"/>
+    <mergeCell ref="C12581:C12582"/>
+    <mergeCell ref="B13100:C13100"/>
+    <mergeCell ref="C13172:C13173"/>
+    <mergeCell ref="C13463:C13464"/>
+    <mergeCell ref="B13291:B13293"/>
+    <mergeCell ref="C12576:C12577"/>
+    <mergeCell ref="B12628:C12628"/>
+    <mergeCell ref="C12635:C12636"/>
+    <mergeCell ref="B12510:C12510"/>
+    <mergeCell ref="B12520:B12522"/>
+    <mergeCell ref="C12405:C12406"/>
+    <mergeCell ref="B12451:C12451"/>
+    <mergeCell ref="C12468:C12469"/>
+    <mergeCell ref="C13056:C13057"/>
+    <mergeCell ref="C12820:C12821"/>
+    <mergeCell ref="B12982:C12982"/>
+    <mergeCell ref="B12994:B12996"/>
+    <mergeCell ref="B12687:C12687"/>
+    <mergeCell ref="B12701:B12703"/>
+    <mergeCell ref="B12697:B12699"/>
+    <mergeCell ref="C12708:C12709"/>
+    <mergeCell ref="C12278:C12279"/>
+    <mergeCell ref="B12333:C12333"/>
+    <mergeCell ref="C12352:C12353"/>
+    <mergeCell ref="C12106:C12107"/>
+    <mergeCell ref="B12156:C12156"/>
+    <mergeCell ref="C12226:C12227"/>
+    <mergeCell ref="C11758:C11759"/>
+    <mergeCell ref="C11866:C11867"/>
+    <mergeCell ref="C12047:C12048"/>
     <mergeCell ref="C8800:C8801"/>
     <mergeCell ref="C11516:C11517"/>
     <mergeCell ref="C11575:C11576"/>
@@ -54612,54 +54549,117 @@
     <mergeCell ref="B8921:B8923"/>
     <mergeCell ref="C8859:C8860"/>
     <mergeCell ref="B8911:C8911"/>
-    <mergeCell ref="C12278:C12279"/>
-    <mergeCell ref="B12333:C12333"/>
-    <mergeCell ref="C12352:C12353"/>
-    <mergeCell ref="C12106:C12107"/>
-    <mergeCell ref="B12156:C12156"/>
-    <mergeCell ref="C12226:C12227"/>
-    <mergeCell ref="C11758:C11759"/>
-    <mergeCell ref="C11866:C11867"/>
-    <mergeCell ref="C12047:C12048"/>
-    <mergeCell ref="C12576:C12577"/>
-    <mergeCell ref="B12628:C12628"/>
-    <mergeCell ref="C12635:C12636"/>
-    <mergeCell ref="B12510:C12510"/>
-    <mergeCell ref="B12520:B12522"/>
-    <mergeCell ref="C12405:C12406"/>
-    <mergeCell ref="B12451:C12451"/>
-    <mergeCell ref="C12468:C12469"/>
-    <mergeCell ref="C13056:C13057"/>
-    <mergeCell ref="C12820:C12821"/>
-    <mergeCell ref="B12982:C12982"/>
-    <mergeCell ref="B12994:B12996"/>
-    <mergeCell ref="B12687:C12687"/>
-    <mergeCell ref="B12701:B12703"/>
-    <mergeCell ref="B12697:B12699"/>
-    <mergeCell ref="C12708:C12709"/>
-    <mergeCell ref="B13631:C13631"/>
-    <mergeCell ref="C13935:C13936"/>
-    <mergeCell ref="B14044:C14044"/>
-    <mergeCell ref="C14166:C14167"/>
-    <mergeCell ref="B14221:C14221"/>
-    <mergeCell ref="C14464:C14465"/>
-    <mergeCell ref="C13223:C13224"/>
-    <mergeCell ref="B13277:C13277"/>
-    <mergeCell ref="C12581:C12582"/>
-    <mergeCell ref="B13100:C13100"/>
-    <mergeCell ref="C13172:C13173"/>
-    <mergeCell ref="C13463:C13464"/>
-    <mergeCell ref="B13291:B13293"/>
-    <mergeCell ref="B14988:C14988"/>
-    <mergeCell ref="B15047:C15047"/>
-    <mergeCell ref="C14816:C14817"/>
-    <mergeCell ref="B14870:C14870"/>
-    <mergeCell ref="C14523:C14524"/>
-    <mergeCell ref="B14516:C14516"/>
-    <mergeCell ref="B14457:C14457"/>
-    <mergeCell ref="B14575:C14575"/>
-    <mergeCell ref="B14585:B14587"/>
-    <mergeCell ref="B14589:B14591"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B1182:C1182"/>
+    <mergeCell ref="B1005:C1005"/>
+    <mergeCell ref="A145:C145"/>
+    <mergeCell ref="A24:C27"/>
+    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="B179:C179"/>
+    <mergeCell ref="B75:B77"/>
+    <mergeCell ref="B1477:C1477"/>
+    <mergeCell ref="B1359:C1359"/>
+    <mergeCell ref="B1300:C1300"/>
+    <mergeCell ref="B887:C887"/>
+    <mergeCell ref="C950:C951"/>
+    <mergeCell ref="B1064:C1064"/>
+    <mergeCell ref="C1248:C1249"/>
+    <mergeCell ref="C367:C368"/>
+    <mergeCell ref="B415:C415"/>
+    <mergeCell ref="B710:C710"/>
+    <mergeCell ref="B828:C828"/>
+    <mergeCell ref="C839:C840"/>
+    <mergeCell ref="C1307:C1308"/>
+    <mergeCell ref="C1314:C1315"/>
+    <mergeCell ref="B1369:B1371"/>
+    <mergeCell ref="B1373:B1375"/>
+    <mergeCell ref="B1123:C1123"/>
+    <mergeCell ref="C2255:C2256"/>
+    <mergeCell ref="B2244:C2244"/>
+    <mergeCell ref="B1949:C1949"/>
+    <mergeCell ref="B1890:C1890"/>
+    <mergeCell ref="B1831:C1831"/>
+    <mergeCell ref="B1772:C1772"/>
+    <mergeCell ref="B1713:C1713"/>
+    <mergeCell ref="C1787:C1788"/>
+    <mergeCell ref="B1654:C1654"/>
+    <mergeCell ref="B1963:B1965"/>
+    <mergeCell ref="B2775:C2775"/>
+    <mergeCell ref="C2838:C2839"/>
+    <mergeCell ref="B2893:C2893"/>
+    <mergeCell ref="B2657:C2657"/>
+    <mergeCell ref="B2716:C2716"/>
+    <mergeCell ref="C2727:C2728"/>
+    <mergeCell ref="C3202:C3203"/>
+    <mergeCell ref="B3188:C3188"/>
+    <mergeCell ref="C3077:C3078"/>
+    <mergeCell ref="C3136:C3137"/>
+    <mergeCell ref="C3195:C3196"/>
+    <mergeCell ref="B3011:C3011"/>
+    <mergeCell ref="B3365:C3365"/>
+    <mergeCell ref="C3675:C3676"/>
+    <mergeCell ref="B3257:B3259"/>
+    <mergeCell ref="B3261:B3263"/>
+    <mergeCell ref="B3247:C3247"/>
+    <mergeCell ref="B4604:C4604"/>
+    <mergeCell ref="B4663:C4663"/>
+    <mergeCell ref="C4726:C4727"/>
+    <mergeCell ref="B3660:C3660"/>
+    <mergeCell ref="B3837:C3837"/>
+    <mergeCell ref="B3896:C3896"/>
+    <mergeCell ref="C4143:C4144"/>
+    <mergeCell ref="B4191:C4191"/>
+    <mergeCell ref="B4014:C4014"/>
+    <mergeCell ref="C4025:C4026"/>
+    <mergeCell ref="B4132:C4132"/>
+    <mergeCell ref="B3851:B3853"/>
+    <mergeCell ref="C5024:C5025"/>
+    <mergeCell ref="B4781:C4781"/>
+    <mergeCell ref="C4969:C4970"/>
+    <mergeCell ref="B4899:C4899"/>
+    <mergeCell ref="C4615:C4616"/>
+    <mergeCell ref="B5135:C5135"/>
+    <mergeCell ref="B5145:B5147"/>
+    <mergeCell ref="B5149:B5151"/>
+    <mergeCell ref="B5076:C5076"/>
+    <mergeCell ref="C5083:C5084"/>
+    <mergeCell ref="C5090:C5091"/>
+    <mergeCell ref="B5607:C5607"/>
+    <mergeCell ref="B5430:C5430"/>
+    <mergeCell ref="B5489:C5489"/>
+    <mergeCell ref="B5548:C5548"/>
+    <mergeCell ref="C5563:C5564"/>
+    <mergeCell ref="B6669:C6669"/>
+    <mergeCell ref="B6787:C6787"/>
+    <mergeCell ref="C6031:C6032"/>
+    <mergeCell ref="B6492:C6492"/>
+    <mergeCell ref="C6503:C6504"/>
+    <mergeCell ref="C6614:C6615"/>
+    <mergeCell ref="B5739:B5741"/>
+    <mergeCell ref="B5725:C5725"/>
+    <mergeCell ref="C8741:C8742"/>
+    <mergeCell ref="B7627:B7629"/>
+    <mergeCell ref="C8502:C8503"/>
+    <mergeCell ref="B8557:C8557"/>
+    <mergeCell ref="B8675:C8675"/>
+    <mergeCell ref="B7613:C7613"/>
+    <mergeCell ref="B5784:C5784"/>
+    <mergeCell ref="B7672:C7672"/>
+    <mergeCell ref="B6020:C6020"/>
+    <mergeCell ref="C6853:C6854"/>
+    <mergeCell ref="C6912:C6913"/>
+    <mergeCell ref="C6971:C6972"/>
+    <mergeCell ref="B6964:C6964"/>
+    <mergeCell ref="C7451:C7452"/>
+    <mergeCell ref="B7436:C7436"/>
+    <mergeCell ref="C7558:C7559"/>
+    <mergeCell ref="B7209:B7211"/>
+    <mergeCell ref="B7318:C7318"/>
+    <mergeCell ref="C6978:C6979"/>
+    <mergeCell ref="B7023:C7023"/>
+    <mergeCell ref="B7033:B7035"/>
+    <mergeCell ref="B7037:B7039"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup scale="79" orientation="portrait" r:id="rId1"/>

</xml_diff>